<commit_message>
add manager name in excel sheet
</commit_message>
<xml_diff>
--- a/scratch/test_export_result.xlsx
+++ b/scratch/test_export_result.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Timesheet Data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timesheet Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -439,16 +439,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -464,25 +465,30 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Manager Name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Hours Worked</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Billable Status</t>
         </is>
@@ -491,33 +497,34 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>T_Kartik</t>
+          <t>T_Raj</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Employee Records</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>API Development</t>
+          <t>H_Saurabh</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Created CRUD endpoints</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="n">
+          <t>Test Limit</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Billable</t>
         </is>
@@ -526,33 +533,918 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>T_Kartik</t>
+          <t>T_Raj</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Employee Records</t>
+          <t>Sample Project</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Database Design</t>
+          <t>M_Priyanka</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Designed employee table schema</t>
+          <t xml:space="preserve">Maintenance </t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
+          <t>I did....</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>T_Raj</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>H_Saurabh</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>T_Raj</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>M_Tejas</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maintenance </t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>...updated ts</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>T_Raj</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>M_Tejas</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>T_Raj</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>H_Saurabh</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>T_Raj</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>H_Saurabh</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>T_Raj</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>H_Saurabh</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>T_Raj</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>H_Saurabh</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>mno</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>T_Raj</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>H_Saurabh</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>mno</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>T_Raj</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>H_Saurabh</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>jkl</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>T_Raj</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>H_Saurabh</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>jkl</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>T_Raj</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>H_Saurabh</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>ghi</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>T_Raj</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>H_Saurabh</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>ghi</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>T_Raj</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>H_Saurabh</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>def</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>T_Raj</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>H_Saurabh</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>def</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>T_Raj</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>H_Saurabh</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>T_Raj</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>H_Saurabh</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>T_Raj</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>H_Saurabh</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Modifications</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>xyz</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>T_Raj</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>H_Saurabh</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Modifications</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>xyz</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>T_Raj</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>H_Saurabh</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Modifications</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>xyz</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>T_Raj</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>H_Saurabh</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Modifications</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>T_Raj</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>H_Saurabh</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Modifications</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>T_Raj</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Payroll System</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>M_Priyanka</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Tax Calculation</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Added tax deduction logic</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="F3" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G25" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>Billable</t>
         </is>
@@ -569,7 +1461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -601,7 +1493,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>18</v>
+        <v>196</v>
       </c>
     </row>
     <row r="5">
@@ -619,42 +1511,72 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Employee Records</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>18</v>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sample Project</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Billability Breakdown</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Hours</t>
-        </is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>170</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Billable</t>
+          <t>Payroll System</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Billability Breakdown</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Hours</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Non-Billable</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B13" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>